<commit_message>
Remove o TikTok e mantém apenas o Instagram
Coleta de 21/10/2026 do Instagram. O painel, a configuração das redes e o README deixam de incluir o TikTok.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/seguidores instagram.xlsx
+++ b/data/seguidores instagram.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\felip\Documents\Seguidores RN\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2168A6E8-BC50-4F92-8CB9-629FCE516548}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7C7C319-9CDE-46EE-8CFB-D092EFF28CBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -365,7 +365,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.7109375" bestFit="1" customWidth="1"/>
@@ -448,6 +448,17 @@
         <v>482758</v>
       </c>
     </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" s="2">
+        <v>46316</v>
+      </c>
+      <c r="B8" s="3">
+        <v>159255</v>
+      </c>
+      <c r="C8" s="3">
+        <v>486530</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>